<commit_message>
Añadir seccion Flexol con los tejidos tecnicos desde PRECIOS/FLEXOL ENERO 2026.xlsx
</commit_message>
<xml_diff>
--- a/precios_catalogo.xlsx
+++ b/precios_catalogo.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G265"/>
+  <dimension ref="A1:G275"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9073,6 +9073,296 @@
       </c>
       <c r="G265" t="inlineStr"/>
     </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>FLX-5201</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>SCREENFLEX (Poliéster) - PL. 5201</t>
+        </is>
+      </c>
+      <c r="C266" t="n">
+        <v>65</v>
+      </c>
+      <c r="D266" t="n">
+        <v>48.75</v>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>Flexol</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr"/>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>FLX-4153</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>SCREENFLEX (Poliéster) - PL. 4153</t>
+        </is>
+      </c>
+      <c r="C267" t="n">
+        <v>62</v>
+      </c>
+      <c r="D267" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>Flexol</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr"/>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>FLX-4155</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>SCREENFLEX (Poliéster) - PL. 4155 (Colores especiales +10%)</t>
+        </is>
+      </c>
+      <c r="C268" t="n">
+        <v>59</v>
+      </c>
+      <c r="D268" t="n">
+        <v>44.25</v>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>Flexol</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr"/>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>FLX-LISBOA</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>LISBOA Opaco</t>
+        </is>
+      </c>
+      <c r="C269" t="n">
+        <v>69</v>
+      </c>
+      <c r="D269" t="n">
+        <v>51.75</v>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>Flexol</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr"/>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>FLX-SHANTUNG</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>SHANTUNG</t>
+        </is>
+      </c>
+      <c r="C270" t="n">
+        <v>48</v>
+      </c>
+      <c r="D270" t="n">
+        <v>36</v>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>Flexol</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr"/>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>FLX-4241</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>SCREENFLEX (Fibra de Vidrio) - FV. 4241</t>
+        </is>
+      </c>
+      <c r="C271" t="n">
+        <v>71</v>
+      </c>
+      <c r="D271" t="n">
+        <v>53.25</v>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>Flexol</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr"/>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>FLX-3903</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>SCREENFLEX (Fibra de Vidrio) - FV. 3903</t>
+        </is>
+      </c>
+      <c r="C272" t="n">
+        <v>68</v>
+      </c>
+      <c r="D272" t="n">
+        <v>51</v>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>Flexol</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr"/>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>FLX-3935</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>SCREENFLEX (Fibra de Vidrio) - FV. 3935</t>
+        </is>
+      </c>
+      <c r="C273" t="n">
+        <v>65</v>
+      </c>
+      <c r="D273" t="n">
+        <v>48.75</v>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>Flexol</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr"/>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>FLX-MALITR</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>MALI Traslúcido</t>
+        </is>
+      </c>
+      <c r="C274" t="n">
+        <v>48</v>
+      </c>
+      <c r="D274" t="n">
+        <v>36</v>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>Flexol</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr"/>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>FLX-MALIOP</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>MALI Opaco</t>
+        </is>
+      </c>
+      <c r="C275" t="n">
+        <v>60</v>
+      </c>
+      <c r="D275" t="n">
+        <v>45</v>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>Flexol</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>